<commit_message>
fix: backport AdverseEvent.code et .outcome (R5) via extensions locales
category est fixé à medication-mishap (code issu de la révision R5 du
CodeSystem partagé adverse-event-category) ; le JDV jdv-origine-effet-
indesirable-cisis migre vers une nouvelle extension "code" (backport
AdverseEvent.code, renommage R5 de event, event neutralisé à 0..0).
outcome est neutralisé à 0..0 (binding Required en R4, incompatible
avec jdv-evolution-cisis) et remplacé par une extension "outcome"
(backport R5, binding Example). Ces deux backports ne sont pas
couverts par l'IG cross-version xver-r5.r4 ; leur ^url suit le format
officiel des extensions de backport (http://hl7.org/fhir/5.0/
StructureDefinition/extension-AdverseEvent.<element>). 365c3ec828060ddd34fc8d85d43782905e69a1d7
</commit_message>
<xml_diff>
--- a/nr-doc-core-adverse-event/ig/StructureDefinition-fr-core-address-insee-code.xlsx
+++ b/nr-doc-core-adverse-event/ig/StructureDefinition-fr-core-address-insee-code.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-30T09:44:31+00:00</t>
+    <t>2026-07-30T14:18:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -349,7 +349,7 @@
     <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
   </si>
   <si>
-    <t>extensible</t>
+    <t>required</t>
   </si>
   <si>
     <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-insee-code|2.2.0</t>

</xml_diff>